<commit_message>
Update test contacts data after dry-run test
</commit_message>
<xml_diff>
--- a/contacts.xlsx
+++ b/contacts.xlsx
@@ -473,12 +473,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Diya Shah</t>
+          <t>Reyansh Joshi</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>+916990177450</t>
+          <t>+916248979493</t>
         </is>
       </c>
     </row>
@@ -488,12 +488,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Aarav Kumar</t>
+          <t>Pooja Reddy</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>+917707709852</t>
+          <t>+917091517602</t>
         </is>
       </c>
     </row>
@@ -503,12 +503,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Saanvi Verma</t>
+          <t>Ishaan Reddy</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>+918108741975</t>
+          <t>+919093650132</t>
         </is>
       </c>
     </row>
@@ -518,12 +518,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Arjun Gupta</t>
+          <t>Riya Rao</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>+917100394655</t>
+          <t>+918072782046</t>
         </is>
       </c>
     </row>
@@ -533,12 +533,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Pooja Mishra</t>
+          <t>Priya Kumar</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>+916727162513</t>
+          <t>+917240117503</t>
         </is>
       </c>
     </row>
@@ -548,12 +548,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Vivaan Desai</t>
+          <t>Diya Iyer</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>+917318883304</t>
+          <t>+918546648031</t>
         </is>
       </c>
     </row>
@@ -563,12 +563,12 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Reyansh Verma</t>
+          <t>Shreya Patel</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>+916383054385</t>
+          <t>+918425181983</t>
         </is>
       </c>
     </row>
@@ -578,12 +578,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Ananya Reddy</t>
+          <t>Ananya Mishra</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+919520206943</t>
+          <t>+916952384532</t>
         </is>
       </c>
     </row>
@@ -593,12 +593,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Vihaan Patel</t>
+          <t>Meera Mehta</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>+918629100144</t>
+          <t>+918607608008</t>
         </is>
       </c>
     </row>
@@ -608,12 +608,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Neha Kumar</t>
+          <t>Vivaan Reddy</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>+916460751638</t>
+          <t>+919641640716</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Initialize Chrome profile for WhatsappBulk application and update test_single.xlsx.
</commit_message>
<xml_diff>
--- a/contacts.xlsx
+++ b/contacts.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -473,12 +473,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Reyansh Joshi</t>
+          <t>Diya Rao</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>+916248979493</t>
+          <t>+918851355857</t>
         </is>
       </c>
     </row>
@@ -488,12 +488,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Pooja Reddy</t>
+          <t>Aarav Mehta</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>+917091517602</t>
+          <t>+918655464251</t>
         </is>
       </c>
     </row>
@@ -503,12 +503,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Ishaan Reddy</t>
+          <t>Shreya Reddy</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>+919093650132</t>
+          <t>+918420394279</t>
         </is>
       </c>
     </row>
@@ -518,12 +518,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Riya Rao</t>
+          <t>Ishaan Gupta</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>+918072782046</t>
+          <t>+917305395384</t>
         </is>
       </c>
     </row>
@@ -533,12 +533,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Priya Kumar</t>
+          <t>Ayaan Shah</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>+917240117503</t>
+          <t>+917827174325</t>
         </is>
       </c>
     </row>
@@ -548,12 +548,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Diya Iyer</t>
+          <t>Krishna Mishra</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>+918546648031</t>
+          <t>+917481799379</t>
         </is>
       </c>
     </row>
@@ -563,12 +563,12 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Shreya Patel</t>
+          <t>Vivaan Joshi</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>+918425181983</t>
+          <t>+918737361071</t>
         </is>
       </c>
     </row>
@@ -578,12 +578,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Ananya Mishra</t>
+          <t>Saanvi Joshi</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+916952384532</t>
+          <t>+917319812628</t>
         </is>
       </c>
     </row>
@@ -593,12 +593,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Meera Mehta</t>
+          <t>Vivaan Iyer</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>+918607608008</t>
+          <t>+917385090924</t>
         </is>
       </c>
     </row>
@@ -608,12 +608,762 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+918766862826</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Aarav Joshi</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+917652427318</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Vihaan Mehta</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+917850624428</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Pooja Reddy</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+916865984668</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Diya Shah</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+916029228782</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Kavya Joshi</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>+916329760667</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Reyansh Gupta</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+916375467330</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Meera Singh</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+919399200856</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Arjun Verma</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+918732518822</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Pooja Rao</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+918174474001</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Sai Mehta</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+917857977131</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Krishna Nair</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+917022861664</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Aditya Sharma</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+918952508043</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Arjun Joshi</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+917285985073</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Diya Reddy</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+918528913850</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Sai Singh</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+916333607345</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Diya Desai</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+918235497696</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Pooja Gupta</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+916667403798</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Riya Reddy</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+919428332642</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Shreya Reddy</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+917698704859</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Krishna Verma</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+918858718508</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Ayaan Mehta</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+918179584557</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Sai Gupta</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+918511226508</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Pooja Rao</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+916774106317</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Riya Shah</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+916566893452</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Meera Rao</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+916135583903</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Riya Mehta</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+919917759032</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Arjun Mehta</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+918123939006</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Vivaan Joshi</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+916599477145</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Kavya Verma</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+919043944063</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Reyansh Joshi</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+917128907446</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Arjun Mishra</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+917594531695</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Saanvi Iyer</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+919791166383</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Ayaan Nair</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+917886571661</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Riya Mehta</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+916400152132</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Krishna Sharma</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+917392176700</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Priya Kumar</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+917146148339</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Priya Singh</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+919279564009</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Diya Rao</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+917456948336</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Krishna Rao</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+919276285017</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
           <t>Vivaan Reddy</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>+919641640716</t>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+918150478670</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Vihaan Mishra</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+919304024997</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Ayaan Mehta</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+918564519547</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Ayaan Mehta</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+916781244006</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Ayaan Iyer</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+916979490761</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Aarav Mehta</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+919836125366</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Aarav Desai</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+917453587460</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Priya Kumar</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+916742170118</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Vivaan Mishra</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>+919285752270</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Aditya Mishra</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>+917702589903</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Meera Desai</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>+918370090903</t>
         </is>
       </c>
     </row>

</xml_diff>